<commit_message>
Add legal & ops compliance drafts; update tracker
Documents (markdown + Word), all drafts for legal/insurance review:
- 08 Privacy Policy (production draft) — fixes live-page gaps: Netlify->Cloudflare,
  adds Schedule Builder + Referral Tracking + demographic-data disclosure
- 09 Terms of Service (production draft) — replaces the beta "test data only" agreement
- 10 Master Services Agreement (skeleton for attorney; a contract, not a web page)
- 11 Acceptable Use Policy
- 12 Business Continuity & Disaster Recovery plan
- 13 Secrets Management policy
- 14 Data access/correction/deletion runbook
Also: Exhibit B correction in 01; tracker updated (22 items in progress, vendor gaps 8->5).

Not legal advice. Lives outside public/ so it is never web-served.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Cohort_Logic_Compliance_Tracker.xlsx
+++ b/compliance/Cohort_Logic_Compliance_Tracker.xlsx
@@ -1550,7 +1550,7 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
@@ -1561,7 +1561,7 @@
       <c r="H11" s="25" t="inlineStr"/>
       <c r="I11" s="25" t="inlineStr">
         <is>
-          <t>Send current privacy.html to counsel.</t>
+          <t>Production draft at compliance/08_Privacy_Policy_DRAFT.md — attorney review, then port to privacy.html (fixes Netlify/Schedule/Referrals/demographics gaps).</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="I16" s="24" t="inlineStr">
         <is>
-          <t>Access/correction/deletion process drafted in 02_...(§5) + 03_...; formalize the request runbook.</t>
+          <t>Runbook drafted at compliance/14_Data_Request_Runbook.md — set turnaround + privacy@ intake.</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2506,7 @@
       </c>
       <c r="F16" s="24" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G16" s="24" t="inlineStr">
@@ -2519,7 +2519,11 @@
           <t>SE-08</t>
         </is>
       </c>
-      <c r="I16" s="24" t="inlineStr"/>
+      <c r="I16" s="24" t="inlineStr">
+        <is>
+          <t>BC/DR plan drafted at compliance/12_Business_Continuity_and_DR_Plan.md — set RPO/RTO; depends on Supabase Pro (SE-07).</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
@@ -2646,7 +2650,7 @@
       <c r="H19" s="25" t="inlineStr"/>
       <c r="I19" s="25" t="inlineStr">
         <is>
-          <t>Formalize the doc.</t>
+          <t>Secrets policy drafted at compliance/13_Secrets_Management.md.</t>
         </is>
       </c>
     </row>
@@ -3245,12 +3249,12 @@
       </c>
       <c r="F14" s="24" t="inlineStr">
         <is>
-          <t>Gap</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="G14" s="24" t="inlineStr">
         <is>
-          <t>Bind policies; keep a COI ready (BI-04/05/07).</t>
+          <t>Michael obtaining cyber + E&amp;O coverage; keep COI ready once bound (BI-04/05/07).</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3476,7 @@
       </c>
       <c r="G20" s="24" t="inlineStr">
         <is>
-          <t>State explicitly in privacy policy + DPA.</t>
+          <t>Explicit no-sale/no-ads/no-secondary-use in privacy draft (08_...); finalize + attorney review.</t>
         </is>
       </c>
     </row>
@@ -3780,7 +3784,7 @@
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
@@ -3791,7 +3795,7 @@
       <c r="H7" s="25" t="inlineStr"/>
       <c r="I7" s="25" t="inlineStr">
         <is>
-          <t>Consult a licensed broker. Not advice.</t>
+          <t>Michael obtaining cyber liability coverage (broker).</t>
         </is>
       </c>
     </row>
@@ -3823,7 +3827,7 @@
       </c>
       <c r="F8" s="24" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G8" s="24" t="inlineStr">
@@ -3834,7 +3838,7 @@
       <c r="H8" s="24" t="inlineStr"/>
       <c r="I8" s="24" t="inlineStr">
         <is>
-          <t>Often bundled with cyber.</t>
+          <t>Michael obtaining technology E&amp;O coverage (broker).</t>
         </is>
       </c>
     </row>
@@ -3866,7 +3870,7 @@
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
@@ -3877,7 +3881,7 @@
       <c r="H9" s="25" t="inlineStr"/>
       <c r="I9" s="25" t="inlineStr">
         <is>
-          <t>Ask the broker to quote as a package.</t>
+          <t>Michael obtaining general liability / BOP (broker).</t>
         </is>
       </c>
     </row>
@@ -3956,7 +3960,7 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G11" s="25" t="inlineStr">
@@ -3967,7 +3971,7 @@
       <c r="H11" s="25" t="inlineStr"/>
       <c r="I11" s="25" t="inlineStr">
         <is>
-          <t>Finalize production ToS.</t>
+          <t>Production ToS draft at compliance/09_Terms_of_Service_DRAFT.md — replaces beta agreement; attorney review then port to terms.html.</t>
         </is>
       </c>
     </row>
@@ -3999,7 +4003,7 @@
       </c>
       <c r="F12" s="24" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G12" s="24" t="inlineStr">
@@ -4010,7 +4014,7 @@
       <c r="H12" s="24" t="inlineStr"/>
       <c r="I12" s="24" t="inlineStr">
         <is>
-          <t>Draft with counsel.</t>
+          <t>MSA skeleton at compliance/10_Master_Services_Agreement_SKELETON.md — attorney to draft; contract doc, not a web page.</t>
         </is>
       </c>
     </row>
@@ -4089,7 +4093,7 @@
       </c>
       <c r="F14" s="24" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G14" s="24" t="inlineStr">
@@ -4100,7 +4104,7 @@
       <c r="H14" s="24" t="inlineStr"/>
       <c r="I14" s="24" t="inlineStr">
         <is>
-          <t>Lightweight; publish alongside ToS.</t>
+          <t>AUP draft at compliance/11_Acceptable_Use_Policy_DRAFT.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Trust page content draft; update tracker
- 15 Trust/Security page content (markdown + Word): product-aware reframe of
  security.html — separates browser-only tools (Class Builder, Schedule Builder,
  nothing stored) from database-backed tools (CICO, Referrals, real student data
  under controls), adds control table, sub-processors, compliance, and a security
  contact. Keeps the honest "not yet" voice.
- Flags to resolve on web-port: PBC-vs-LLC entity label in footer, dead Terms/DPA
  links, confirm US-region + encryption-at-rest wording before publishing.
- Tracker: PR-10 in progress (23 total in progress); entity-discrepancy note on BI-01/VQ-01.

Draft content for a later website batch; live security.html not changed.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Cohort_Logic_Compliance_Tracker.xlsx
+++ b/compliance/Cohort_Logic_Compliance_Tracker.xlsx
@@ -2884,7 +2884,7 @@
       </c>
       <c r="G4" s="24" t="inlineStr">
         <is>
-          <t>Document entity + EIN in one place (BI-01/02).</t>
+          <t>Confirm entity/EIN (footer 'PBC' vs LLC discrepancy) + document in one place.</t>
         </is>
       </c>
     </row>
@@ -3662,7 +3662,7 @@
       <c r="H4" s="24" t="inlineStr"/>
       <c r="I4" s="24" t="inlineStr">
         <is>
-          <t>Confirm from formation records (an LLC likely already exists).</t>
+          <t>Confirm exact legal entity — security.html footer says 'PBC', other materials imply LLC; make consistent.</t>
         </is>
       </c>
     </row>
@@ -4775,7 +4775,7 @@
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G13" s="25" t="inlineStr">
@@ -4790,7 +4790,7 @@
       </c>
       <c r="I13" s="25" t="inlineStr">
         <is>
-          <t>Publish once sub-processor DPAs are signed.</t>
+          <t>Trust page content drafted at compliance/15_Trust_Page_Content.md — product-aware reframe; port to security.html in website batch.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scope compliance to Phase 1 launch (Class Builder + Schedule Builder only)
Strategic decision: go to market with the two browser-only products only; defer
CICO + Referral Tracking (and their student-data compliance burden) to Phase 2
until product-market fit is confirmed. Both launch products store NO student data
server-side, which collapses most FERPA/state-law/breach obligations to Phase 2.

- 16 Go-To-Market Scope memo (new): the decision, why it slashes the launch burden,
  the Phase 1 short list, and a Phase 1/2 map of every existing doc.
- Tracker: added a Phase column to every tab (46 Phase 1 / 10 Phase 2), a Phase-1
  launch-focus block on the Dashboard, and a scope note on Start Here.
- Scope banners on 08 (privacy) and 15 (trust page) so they aren't misleading in
  isolation; offered a lean Phase-1 privacy/trust rewrite.

Docs are drafts for review; not legal advice; outside public/ (never web-served).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Cohort_Logic_Compliance_Tracker.xlsx
+++ b/compliance/Cohort_Logic_Compliance_Tracker.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -118,8 +118,23 @@
       <color rgb="009C0006"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0044546A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="008a6a18"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -161,6 +176,16 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF0F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBF3D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -188,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -256,6 +281,27 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -711,7 +757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -725,113 +771,127 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="B3" s="2" t="inlineStr">
+    <row r="2" ht="44" customHeight="1">
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>SCOPE (2026-07-21): Launching Class Builder + Schedule Builder only (browser-only, no student data stored). CICO + Referral Tracking = Phase 2. Each item is tagged Phase 1 / Phase 2. See compliance/16_Go_To_Market_Scope.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="45" customHeight="1">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="45" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>A single living plan to get Cohort Logic production-ready to sell to schools nationwide — covering FERPA &amp; student-data privacy, security hardening, business/legal/insurance, the questionnaire districts will send you, and the product gaps in between.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="2" t="inlineStr">
+    <row r="6"/>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>How the tabs work</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>•  Dashboard — live rollup: how many items per workstream are done / in progress / not started, and how many P0 (must-have) items remain.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>•  FERPA &amp; Privacy, Security &amp; Infra, Business &amp; Insurance, Product &amp; Go-Live — the working checklists. Each row has an ID, priority, status, owner, and next action.</t>
+          <t>•  Dashboard — live rollup: how many items per workstream are done / in progress / not started, and how many P0 (must-have) items remain.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="3" t="inlineStr">
         <is>
+          <t>•  FERPA &amp; Privacy, Security &amp; Infra, Business &amp; Insurance, Product &amp; Go-Live — the working checklists. Each row has an ID, priority, status, owner, and next action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
           <t>•  School Vendor Q&amp;A — the recurring questions procurement/IT send, each with a prepared answer, the evidence, and a readiness rating (Ready / Partial / Gap).</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="2" t="inlineStr">
+    <row r="11"/>
+    <row r="12" ht="60" customHeight="1">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>How we'll manage it</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1">
-      <c r="B12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>This is the tracker I (Claude) maintain for you. Tell me things like “mark SE-07 done,” “what are my open P0 items?,” “add a task for X,” or “what do I still owe a district that just sent a questionnaire?” — and I'll update the file and re-share. IDs (FE-/SE-/VQ-/BI-/PR-) are stable handles for that.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="2" t="inlineStr">
+    <row r="14"/>
+    <row r="15" ht="30" customHeight="1">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Status values (dropdowns)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Checklists: Not started · In progress · Blocked · Done · N/A          Vendor Q&amp;A: Ready · Partial · Gap</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
+          <t>Checklists: Not started · In progress · Blocked · Done · N/A          Vendor Q&amp;A: Ready · Partial · Gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
           <t>Priority: P0 = must-have before selling · P1 = needed early · P2 = important, can follow</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="2" t="inlineStr">
+    <row r="18"/>
+    <row r="19" ht="75" customHeight="1">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>The fastest path to a sellable posture (suggested first moves)</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="75" customHeight="1">
-      <c r="B19" s="3" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>1. Upgrade Supabase to Pro + verify backups (SE-07/08).   2. Sign the Supabase &amp; Cloudflare DPAs and publish a sub-processor list (FE-05).   3. Bind cyber + E&amp;O insurance (BI-04/05).   4. Get a lawyer-reviewed DPA/NDPA template and finalize ToS (FE-02/03, BI-08).   5. Write the data map, retention policy and incident-response/breach plan (FE-04/07/12, SE-12).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="4" t="inlineStr">
+    <row r="21"/>
+    <row r="22" ht="60" customHeight="1">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Important disclaimer</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1">
-      <c r="B22" s="5" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>This tracker is an organizational tool, not legal, insurance, or financial advice. FERPA/state-law, contract, and insurance items must be reviewed by a licensed attorney and a licensed insurance broker before you rely on them. Rows marked “Attorney” or “Broker” as owner are flagged precisely because they need a professional.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="6" t="inlineStr">
+    <row r="24"/>
+    <row r="25">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Last updated by Claude: 2026-07-21</t>
         </is>
@@ -851,7 +911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1117,12 +1177,77 @@
         </is>
       </c>
     </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t>Phase 1 launch focus — Class Builder + Schedule Builder (no student data stored)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Phase 1 items</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>% Phase 1 done</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="28">
+        <f>COUNTIF('FERPA &amp; Privacy'!$J$4:$J$200,"Phase 1")+COUNTIF('Security &amp; Infra'!$J$4:$J$200,"Phase 1")+COUNTIF('Business &amp; Insurance'!$J$4:$J$200,"Phase 1")+COUNTIF('Product &amp; Go-Live'!$J$4:$J$200,"Phase 1")</f>
+        <v/>
+      </c>
+      <c r="B18" s="28">
+        <f>COUNTIFS('FERPA &amp; Privacy'!$J$4:$J$200,"Phase 1",'FERPA &amp; Privacy'!$F$4:$F$200,"Done")+COUNTIFS('Security &amp; Infra'!$J$4:$J$200,"Phase 1",'Security &amp; Infra'!$F$4:$F$200,"Done")+COUNTIFS('Business &amp; Insurance'!$J$4:$J$200,"Phase 1",'Business &amp; Insurance'!$F$4:$F$200,"Done")+COUNTIFS('Product &amp; Go-Live'!$J$4:$J$200,"Phase 1",'Product &amp; Go-Live'!$F$4:$F$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="C18" s="28">
+        <f>COUNTIFS('FERPA &amp; Privacy'!$J$4:$J$200,"Phase 1",'FERPA &amp; Privacy'!$F$4:$F$200,"In progress")+COUNTIFS('Security &amp; Infra'!$J$4:$J$200,"Phase 1",'Security &amp; Infra'!$F$4:$F$200,"In progress")+COUNTIFS('Business &amp; Insurance'!$J$4:$J$200,"Phase 1",'Business &amp; Insurance'!$F$4:$F$200,"In progress")+COUNTIFS('Product &amp; Go-Live'!$J$4:$J$200,"Phase 1",'Product &amp; Go-Live'!$F$4:$F$200,"In progress")</f>
+        <v/>
+      </c>
+      <c r="D18" s="28">
+        <f>COUNTIFS('FERPA &amp; Privacy'!$J$4:$J$200,"Phase 1",'FERPA &amp; Privacy'!$F$4:$F$200,"Not started")+COUNTIFS('Security &amp; Infra'!$J$4:$J$200,"Phase 1",'Security &amp; Infra'!$F$4:$F$200,"Not started")+COUNTIFS('Business &amp; Insurance'!$J$4:$J$200,"Phase 1",'Business &amp; Insurance'!$F$4:$F$200,"Not started")+COUNTIFS('Product &amp; Go-Live'!$J$4:$J$200,"Phase 1",'Product &amp; Go-Live'!$F$4:$F$200,"Not started")</f>
+        <v/>
+      </c>
+      <c r="E18" s="29">
+        <f>IFERROR(B18/A18,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>Phase 2 (CICO / Referral Tracking) is deferred until product-market fit — see the Go-To-Market Scope memo (compliance/16).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="B14:G14"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A19:G19"/>
     <mergeCell ref="A11:G11"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1134,7 +1259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:J219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1146,6 +1271,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1208,6 +1334,11 @@
           <t>Next action / notes</t>
         </is>
       </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
@@ -1251,6 +1382,11 @@
           <t>Draft memo at compliance/03_FERPA_School_Official_Posture.md — needs attorney review.</t>
         </is>
       </c>
+      <c r="J4" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="25" t="inlineStr">
@@ -1298,6 +1434,11 @@
           <t>DPA/NDPA readiness at compliance/07_DPA_and_NDPA_Readiness.md — attorney to produce own-paper DPA/MSA.</t>
         </is>
       </c>
+      <c r="J5" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
@@ -1345,6 +1486,11 @@
           <t>NDPA v2.2 plan in compliance/07_... — join SDPC, prep Exhibit A/B/F, sign Exhibit E (piggyback).</t>
         </is>
       </c>
+      <c r="J6" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
@@ -1388,6 +1534,11 @@
           <t>Data map drafted at compliance/01_Data_Inventory_and_Data_Map.md — confirm audit_log PII + Supabase US region.</t>
         </is>
       </c>
+      <c r="J7" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
@@ -1431,6 +1582,11 @@
           <t>Sign Supabase DPA; get Cloudflare DPA; publish list on the trust page.</t>
         </is>
       </c>
+      <c r="J8" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
@@ -1474,6 +1630,11 @@
           <t>Verify Supabase project region in the dashboard; capture attestation.</t>
         </is>
       </c>
+      <c r="J9" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
@@ -1521,6 +1682,11 @@
           <t>Policy drafted at compliance/02_Data_Retention_and_Deletion_Policy.md — set [DECIDE] windows; verify wipe covers referrals + audit_log.</t>
         </is>
       </c>
+      <c r="J10" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
@@ -1564,6 +1730,11 @@
           <t>Production draft at compliance/08_Privacy_Policy_DRAFT.md — attorney review, then port to privacy.html (fixes Netlify/Schedule/Referrals/demographics gaps).</t>
         </is>
       </c>
+      <c r="J11" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
@@ -1607,6 +1778,11 @@
           <t>Reflect in privacy policy + DPA.</t>
         </is>
       </c>
+      <c r="J12" s="32" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="25" t="inlineStr">
@@ -1650,6 +1826,11 @@
           <t>State matrix at compliance/06_State_Student_Privacy_Matrix.md — confirm [VERIFY] statute cites/timelines with counsel.</t>
         </is>
       </c>
+      <c r="J13" s="32" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
@@ -1697,6 +1878,11 @@
           <t>Only if pursuing the NY market.</t>
         </is>
       </c>
+      <c r="J14" s="32" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="25" t="inlineStr">
@@ -1740,6 +1926,11 @@
           <t>Breach policy at compliance/05_Data_Breach_Notification_Policy.md — 72h default / 7-day hard ceiling.</t>
         </is>
       </c>
+      <c r="J15" s="32" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="24" t="inlineStr">
@@ -1787,6 +1978,11 @@
           <t>Runbook drafted at compliance/14_Data_Request_Runbook.md — set turnaround + privacy@ intake.</t>
         </is>
       </c>
+      <c r="J16" s="32" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
@@ -1830,7 +2026,214 @@
           <t>Document the policy now so there is something to point to.</t>
         </is>
       </c>
-    </row>
+      <c r="J17" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
@@ -1861,12 +2264,15 @@
       <formula>"P2"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="F4:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Blocked,Done,N/A"</formula1>
     </dataValidation>
     <dataValidation sqref="E4:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P0,P1,P2"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J4:J200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Phase 1,Phase 2"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1879,7 +2285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:J219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1891,6 +2297,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1953,6 +2360,11 @@
           <t>Next action / notes</t>
         </is>
       </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
@@ -1996,6 +2408,11 @@
           <t>Verified daily by the security-compliance agent.</t>
         </is>
       </c>
+      <c r="J4" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="25" t="inlineStr">
@@ -2039,6 +2456,11 @@
           <t>In place.</t>
         </is>
       </c>
+      <c r="J5" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
@@ -2082,6 +2504,11 @@
           <t>Verified live by the security agent.</t>
         </is>
       </c>
+      <c r="J6" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
@@ -2129,6 +2556,11 @@
           <t>MFA is available but enrollment is not yet mandatory — see SE-05.</t>
         </is>
       </c>
+      <c r="J7" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
@@ -2172,6 +2604,11 @@
           <t>Flip admin-mfa.js from soft reminder to hard enforcement.</t>
         </is>
       </c>
+      <c r="J8" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
@@ -2215,6 +2652,11 @@
           <t>This agent.</t>
         </is>
       </c>
+      <c r="J9" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
@@ -2258,6 +2700,11 @@
           <t>Already flagged in CLAUDE.md pending list.</t>
         </is>
       </c>
+      <c r="J10" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
@@ -2305,6 +2752,11 @@
           <t>Document the restore runbook.</t>
         </is>
       </c>
+      <c r="J11" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
@@ -2348,6 +2800,11 @@
           <t>Capture Supabase/AWS attestation language.</t>
         </is>
       </c>
+      <c r="J12" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="25" t="inlineStr">
@@ -2391,6 +2848,11 @@
           <t>Get quotes; schedule the first test.</t>
         </is>
       </c>
+      <c r="J13" s="32" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
@@ -2434,6 +2896,11 @@
           <t>Add to CI / the pre-deploy gate.</t>
         </is>
       </c>
+      <c r="J14" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="25" t="inlineStr">
@@ -2477,6 +2944,11 @@
           <t>IR plan drafted at compliance/04_Incident_Response_Plan.md — fill [FILL] counsel/insurer/provider contacts.</t>
         </is>
       </c>
+      <c r="J15" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="24" t="inlineStr">
@@ -2524,6 +2996,11 @@
           <t>BC/DR plan drafted at compliance/12_Business_Continuity_and_DR_Plan.md — set RPO/RTO; depends on Supabase Pro (SE-07).</t>
         </is>
       </c>
+      <c r="J16" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
@@ -2567,6 +3044,11 @@
           <t>e.g. UptimeRobot / BetterStack + a hosted status page.</t>
         </is>
       </c>
+      <c r="J17" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="24" t="inlineStr">
@@ -2610,6 +3092,11 @@
           <t>Supabase Auth settings toggle.</t>
         </is>
       </c>
+      <c r="J18" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="25" t="inlineStr">
@@ -2653,6 +3140,11 @@
           <t>Secrets policy drafted at compliance/13_Secrets_Management.md.</t>
         </is>
       </c>
+      <c r="J19" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="24" t="inlineStr">
@@ -2696,6 +3188,11 @@
           <t>Decision item; consider Vanta/Drata when revenue supports it.</t>
         </is>
       </c>
+      <c r="J20" s="32" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="25" t="inlineStr">
@@ -2739,7 +3236,210 @@
           <t>Configure WAF rules.</t>
         </is>
       </c>
-    </row>
+      <c r="J21" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
@@ -2770,12 +3470,15 @@
       <formula>"P2"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="F4:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Blocked,Done,N/A"</formula1>
     </dataValidation>
     <dataValidation sqref="E4:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P0,P1,P2"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J4:J200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Phase 1,Phase 2"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2788,7 +3491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:H219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2798,6 +3501,7 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2850,6 +3554,11 @@
           <t>Action to be answer-ready</t>
         </is>
       </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
@@ -2887,6 +3596,11 @@
           <t>Confirm entity/EIN (footer 'PBC' vs LLC discrepancy) + document in one place.</t>
         </is>
       </c>
+      <c r="H4" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="25" t="inlineStr">
@@ -2924,6 +3638,11 @@
           <t>Data map drafted (01_...); finalize + confirm flags.</t>
         </is>
       </c>
+      <c r="H5" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
@@ -2961,6 +3680,11 @@
           <t>Confirm + document region.</t>
         </is>
       </c>
+      <c r="H6" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
@@ -2998,6 +3722,11 @@
           <t>Obtain at-rest attestation.</t>
         </is>
       </c>
+      <c r="H7" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
@@ -3035,6 +3764,11 @@
           <t>Note that mandatory MFA is in progress (SE-05).</t>
         </is>
       </c>
+      <c r="H8" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
@@ -3072,6 +3806,11 @@
           <t>Sub-processor list drafted (01_...); sign Supabase + Cloudflare DPAs to close.</t>
         </is>
       </c>
+      <c r="H9" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
@@ -3109,6 +3848,11 @@
           <t>Retention/deletion policy drafted (02_...); set windows + verify wipe scope.</t>
         </is>
       </c>
+      <c r="H10" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
@@ -3146,6 +3890,11 @@
           <t>Breach policy (05_...) + IR plan (04_...) drafted; fill contacts to reach Ready.</t>
         </is>
       </c>
+      <c r="H11" s="32" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
@@ -3183,6 +3932,11 @@
           <t>FERPA posture (03_...) + state matrix (06_...) drafted; needs counsel-reviewed statements.</t>
         </is>
       </c>
+      <c r="H12" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="25" t="inlineStr">
@@ -3220,6 +3974,11 @@
           <t>NDPA readiness brief (07_...) drafted; join SDPC + have signable template to reach Ready.</t>
         </is>
       </c>
+      <c r="H13" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
@@ -3257,6 +4016,11 @@
           <t>Michael obtaining cyber + E&amp;O coverage; keep COI ready once bound (BI-04/05/07).</t>
         </is>
       </c>
+      <c r="H14" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="25" t="inlineStr">
@@ -3294,6 +4058,11 @@
           <t>Pen test first; SOC 2 as a later roadmap item.</t>
         </is>
       </c>
+      <c r="H15" s="32" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="24" t="inlineStr">
@@ -3331,6 +4100,11 @@
           <t>Commission an accessibility audit + VPAT.</t>
         </is>
       </c>
+      <c r="H16" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
@@ -3368,6 +4142,11 @@
           <t>Roadmap SSO/rostering — a major K-12 adoption factor.</t>
         </is>
       </c>
+      <c r="H17" s="32" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="24" t="inlineStr">
@@ -3405,6 +4184,11 @@
           <t>Define SLA + support commitments.</t>
         </is>
       </c>
+      <c r="H18" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="25" t="inlineStr">
@@ -3442,6 +4226,11 @@
           <t>Document the policy (scales with hiring).</t>
         </is>
       </c>
+      <c r="H19" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="24" t="inlineStr">
@@ -3479,6 +4268,11 @@
           <t>Explicit no-sale/no-ads/no-secondary-use in privacy draft (08_...); finalize + attorney review.</t>
         </is>
       </c>
+      <c r="H20" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="A21" s="25" t="inlineStr">
@@ -3516,7 +4310,210 @@
           <t>Gather references/testimonials from pilots.</t>
         </is>
       </c>
-    </row>
+      <c r="H21" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
@@ -3533,9 +4530,12 @@
       <formula>"Gap"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="F4:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Ready,Partial,Gap,N/A"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H4:H200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Phase 1,Phase 2"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3548,7 +4548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:J219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3560,6 +4560,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3622,6 +4623,11 @@
           <t>Next action / notes</t>
         </is>
       </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
@@ -3665,6 +4671,11 @@
           <t>Confirm exact legal entity — security.html footer says 'PBC', other materials imply LLC; make consistent.</t>
         </is>
       </c>
+      <c r="J4" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="25" t="inlineStr">
@@ -3712,6 +4723,11 @@
           <t>Keep a signed W-9 on file.</t>
         </is>
       </c>
+      <c r="J5" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
@@ -3755,6 +4771,11 @@
           <t>Confirm (bookkeeping already underway).</t>
         </is>
       </c>
+      <c r="J6" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
@@ -3798,6 +4819,11 @@
           <t>Michael obtaining cyber liability coverage (broker).</t>
         </is>
       </c>
+      <c r="J7" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
@@ -3841,6 +4867,11 @@
           <t>Michael obtaining technology E&amp;O coverage (broker).</t>
         </is>
       </c>
+      <c r="J8" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
@@ -3884,6 +4915,11 @@
           <t>Michael obtaining general liability / BOP (broker).</t>
         </is>
       </c>
+      <c r="J9" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
@@ -3931,6 +4967,11 @@
           <t>Store a current COI to attach to questionnaires.</t>
         </is>
       </c>
+      <c r="J10" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
@@ -3974,6 +5015,11 @@
           <t>Production ToS draft at compliance/09_Terms_of_Service_DRAFT.md — replaces beta agreement; attorney review then port to terms.html.</t>
         </is>
       </c>
+      <c r="J11" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
@@ -4017,6 +5063,11 @@
           <t>MSA skeleton at compliance/10_Master_Services_Agreement_SKELETON.md — attorney to draft; contract doc, not a web page.</t>
         </is>
       </c>
+      <c r="J12" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="25" t="inlineStr">
@@ -4064,6 +5115,11 @@
           <t>Keep the legal and product copies in sync.</t>
         </is>
       </c>
+      <c r="J13" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
@@ -4107,6 +5163,11 @@
           <t>AUP draft at compliance/11_Acceptable_Use_Policy_DRAFT.md.</t>
         </is>
       </c>
+      <c r="J14" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="25" t="inlineStr">
@@ -4150,6 +5211,11 @@
           <t>Optional; search availability first.</t>
         </is>
       </c>
+      <c r="J15" s="32" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="24" t="inlineStr">
@@ -4193,6 +5259,11 @@
           <t>Handle as encountered.</t>
         </is>
       </c>
+      <c r="J16" s="32" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
@@ -4236,7 +5307,214 @@
           <t>Have someone on call before the first deal.</t>
         </is>
       </c>
-    </row>
+      <c r="J17" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
@@ -4267,12 +5545,15 @@
       <formula>"P2"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="F4:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Blocked,Done,N/A"</formula1>
     </dataValidation>
     <dataValidation sqref="E4:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P0,P1,P2"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J4:J200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Phase 1,Phase 2"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4285,7 +5566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4297,6 +5578,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4359,6 +5641,11 @@
           <t>Next action / notes</t>
         </is>
       </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
@@ -4402,6 +5689,11 @@
           <t>Design plans + checkout + webhooks.</t>
         </is>
       </c>
+      <c r="J4" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="25" t="inlineStr">
@@ -4445,6 +5737,11 @@
           <t>Admin tooling exists; formalize the flow.</t>
         </is>
       </c>
+      <c r="J5" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
@@ -4488,6 +5785,11 @@
           <t>e.g. email + help desk; publish response targets.</t>
         </is>
       </c>
+      <c r="J6" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
@@ -4531,6 +5833,11 @@
           <t>Start with top workflows per product.</t>
         </is>
       </c>
+      <c r="J7" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
@@ -4574,6 +5881,11 @@
           <t>Feeds VQ-13.</t>
         </is>
       </c>
+      <c r="J8" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
@@ -4617,6 +5929,11 @@
           <t>Feeds VQ-14; sequence after billing.</t>
         </is>
       </c>
+      <c r="J9" s="32" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
@@ -4660,6 +5977,11 @@
         </is>
       </c>
       <c r="I10" s="24" t="inlineStr"/>
+      <c r="J10" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
@@ -4703,6 +6025,11 @@
           <t>Already in CLAUDE.md pending.</t>
         </is>
       </c>
+      <c r="J11" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
@@ -4746,6 +6073,11 @@
           <t>Confirm tiers before wiring Stripe.</t>
         </is>
       </c>
+      <c r="J12" s="30" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="25" t="inlineStr">
@@ -4793,7 +6125,218 @@
           <t>Trust page content drafted at compliance/15_Trust_Page_Content.md — product-aware reframe; port to security.html in website batch.</t>
         </is>
       </c>
-    </row>
+      <c r="J13" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
@@ -4824,13 +6367,16 @@
       <formula>"P2"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="F4:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Blocked,Done,N/A"</formula1>
     </dataValidation>
     <dataValidation sqref="E4:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P0,P1,P2"</formula1>
     </dataValidation>
+    <dataValidation sqref="J4:J200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Phase 1,Phase 2"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add lean Phase-1 launch privacy policy and trust page
Clean, launch-ready versions scoped to Class Builder + Schedule Builder only,
leading with "student data never reaches our servers":
- 17 Privacy Policy (Phase 1 launch) — covers only staff accounts + anonymous
  analytics; no CICO/Referrals/demographics. Supersedes 08 for launch (08 kept
  as the Phase-2 baseline).
- 18 Trust page (Phase 1 launch) — browser-only story, control table, sub-processors,
  security contact; keeps the honest "not yet" voice. Supersedes 15 for launch.
- Tracker: FE-08/PR-10 point to the launch versions; VQ-02 now Ready.

Drafts for attorney review; not legal advice; outside public/ (never web-served).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Cohort_Logic_Compliance_Tracker.xlsx
+++ b/compliance/Cohort_Logic_Compliance_Tracker.xlsx
@@ -757,7 +757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="B1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -778,7 +778,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="45" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -793,7 +792,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="2" t="inlineStr">
         <is>
@@ -822,7 +820,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="60" customHeight="1">
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -837,7 +834,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -859,7 +855,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="75" customHeight="1">
       <c r="B19" s="2" t="inlineStr">
         <is>
@@ -874,7 +869,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="60" customHeight="1">
       <c r="B22" s="4" t="inlineStr">
         <is>
@@ -889,7 +883,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="B25" s="6" t="inlineStr">
         <is>
@@ -1259,7 +1252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J219"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1727,7 +1720,7 @@
       <c r="H11" s="25" t="inlineStr"/>
       <c r="I11" s="25" t="inlineStr">
         <is>
-          <t>Production draft at compliance/08_Privacy_Policy_DRAFT.md — attorney review, then port to privacy.html (fixes Netlify/Schedule/Referrals/demographics gaps).</t>
+          <t>LAUNCH version at compliance/17_Privacy_Policy_Phase1_LAUNCH.md (lean, no student data); 08 kept as Phase-2 baseline. Attorney review then port.</t>
         </is>
       </c>
       <c r="J11" s="31" t="inlineStr">
@@ -2032,208 +2025,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
@@ -2285,7 +2076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J219"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3242,204 +3033,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
@@ -3491,7 +3084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H219"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3630,12 +3223,12 @@
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>Data map drafted (01_...); finalize + confirm flags.</t>
+          <t>Launch products store NO student data server-side (only staff accounts + anonymous analytics) — clean answer; see 17_/18_.</t>
         </is>
       </c>
       <c r="H5" s="31" t="inlineStr">
@@ -4316,204 +3909,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
@@ -4548,7 +3943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J219"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5313,208 +4708,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
@@ -5566,7 +4759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J219"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6122,7 +5315,7 @@
       </c>
       <c r="I13" s="25" t="inlineStr">
         <is>
-          <t>Trust page content drafted at compliance/15_Trust_Page_Content.md — product-aware reframe; port to security.html in website batch.</t>
+          <t>LAUNCH version at compliance/18_Trust_Page_Phase1_LAUNCH.md (browser-only story); 15 kept for Phase 2. Port to security.html in web batch.</t>
         </is>
       </c>
       <c r="J13" s="31" t="inlineStr">
@@ -6131,212 +5324,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
Add recommended-defaults sheet, Stripe billing plan, and signable DPA template
- 20 Recommended Defaults & Decisions — a value for every [DECIDE]/[FILL]/[CONFIRM]
  blank across the docs, split into approve / you-supply / confirm-externally.
- 21 Stripe Billing Plan — per-school subscriptions via Stripe Checkout + Supabase
  Edge Functions; reconciles with the existing subscriptions ledger; gating via
  enabled_products; secrets kept server-side. Design + decisions before code.
- 22 Data Processing Agreement (short-form template) — signable fill-in-the-blanks
  DPA reflecting the no-student-data-stored posture (near-empty data schedule).
- Tracker: PR-01 in progress (plan); FE-02 points to the signable DPA.

Drafts/plans for review; not legal advice; outside public/ (never web-served).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Cohort_Logic_Compliance_Tracker.xlsx
+++ b/compliance/Cohort_Logic_Compliance_Tracker.xlsx
@@ -1272,7 +1272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J219"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1444,7 +1444,7 @@
       </c>
       <c r="I5" s="25" t="inlineStr">
         <is>
-          <t>DPA/NDPA readiness at compliance/07_DPA_and_NDPA_Readiness.md — attorney to produce own-paper DPA/MSA.</t>
+          <t>Signable short-form DPA at compliance/22_...; readiness/NDPA context in 07_. Attorney review before use.</t>
         </is>
       </c>
       <c r="J5" s="31" t="inlineStr">
@@ -2097,207 +2097,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
@@ -5141,7 +4940,7 @@
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G4" s="24" t="inlineStr">
@@ -5152,7 +4951,7 @@
       <c r="H4" s="24" t="inlineStr"/>
       <c r="I4" s="24" t="inlineStr">
         <is>
-          <t>Design plans + checkout + webhooks.</t>
+          <t>Implementation plan at compliance/21_Stripe_Billing_Plan.md (Supabase Edge Functions + Stripe Checkout). Needs pricing decision + code batch.</t>
         </is>
       </c>
       <c r="J4" s="30" t="inlineStr">

</xml_diff>

<commit_message>
Correct entity to Cohort Logic, LLC; add Stripe billing DB migration
- Entity confirmed by owner as Cohort Logic, LLC (not "PBC" — a PBC is a different
  entity type). Corrected across compliance docs 16/17/18/20/22 and tracker
  BI-01/VQ-01. NOTE: the live site footers say "Cohort Logic, PBC" on 10 pages
  (index, pricing, products, security, contact, resources, class-builder,
  schedule-builder [+JSON-LD], balanced-classes, prepare-student-roster) — left
  unchanged pending the reviewed website batch.
- supabase/migrations/stripe_billing.sql: additive Stripe linkage columns on
  subscriptions (customer/subscription/price ids, current_period_end,
  cancel_at_period_end) + unique indexes. Webhook (service-role) is the single
  writer; RLS unchanged. Run in the SQL editor when ready.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Cohort_Logic_Compliance_Tracker.xlsx
+++ b/compliance/Cohort_Logic_Compliance_Tracker.xlsx
@@ -3258,7 +3258,7 @@
       </c>
       <c r="G4" s="24" t="inlineStr">
         <is>
-          <t>Confirm entity/EIN (footer 'PBC' vs LLC discrepancy) + document in one place.</t>
+          <t>Entity = Cohort Logic, LLC (confirmed). Document EIN/W-9; fix footer 'PBC'-&gt;'LLC' in website batch.</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -4124,7 +4124,7 @@
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G4" s="24" t="inlineStr">
@@ -4135,7 +4135,7 @@
       <c r="H4" s="24" t="inlineStr"/>
       <c r="I4" s="24" t="inlineStr">
         <is>
-          <t>Confirm exact legal entity — security.html footer says 'PBC', other materials imply LLC; make consistent.</t>
+          <t>Entity = Cohort Logic, LLC (confirmed by owner). Site footers wrongly say 'PBC' on 10 pages — fix in website batch. Still: document EIN/W-9 (BI-02).</t>
         </is>
       </c>
       <c r="J4" s="30" t="inlineStr">

</xml_diff>